<commit_message>
Fix export so muon giao vien
</commit_message>
<xml_diff>
--- a/public/system/export/borrowdevice.xlsx
+++ b/public/system/export/borrowdevice.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="19">
   <si>
     <t>STT</t>
   </si>
@@ -54,19 +54,10 @@
     <t>GHI CHÚ</t>
   </si>
   <si>
-    <t>Quản Trị Viên</t>
-  </si>
-  <si>
     <t>Giáo Viên</t>
   </si>
   <si>
-    <t>Hoàn thành tốt</t>
-  </si>
-  <si>
     <t>x</t>
-  </si>
-  <si>
-    <t>Thể dục - Quốc phòng-AN</t>
   </si>
   <si>
     <t>MỤC ĐÍCH
@@ -279,20 +270,20 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -520,34 +511,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="15" customHeight="1">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="19"/>
+      <c r="B1" s="20"/>
       <c r="C1" s="9"/>
       <c r="D1" s="9"/>
-      <c r="E1" s="20" t="s">
+      <c r="E1" s="23" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-      <c r="I1" s="20"/>
+      <c r="F1" s="23"/>
+      <c r="G1" s="23"/>
+      <c r="H1" s="23"/>
+      <c r="I1" s="23"/>
     </row>
     <row r="2" spans="1:9" ht="15" customHeight="1">
-      <c r="A2" s="19" t="s">
+      <c r="A2" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="19"/>
+      <c r="B2" s="20"/>
       <c r="C2" s="9"/>
       <c r="D2" s="9"/>
-      <c r="E2" s="20" t="s">
+      <c r="E2" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="20"/>
-      <c r="G2" s="20"/>
-      <c r="H2" s="20"/>
-      <c r="I2" s="20"/>
+      <c r="F2" s="23"/>
+      <c r="G2" s="23"/>
+      <c r="H2" s="23"/>
+      <c r="I2" s="23"/>
     </row>
     <row r="3" spans="1:9" ht="15" customHeight="1">
       <c r="A3" s="1"/>
@@ -561,17 +552,17 @@
       <c r="I3" s="10"/>
     </row>
     <row r="4" spans="1:9" ht="18" customHeight="1">
-      <c r="A4" s="22" t="s">
-        <v>21</v>
-      </c>
-      <c r="B4" s="23"/>
-      <c r="C4" s="23"/>
-      <c r="D4" s="23"/>
-      <c r="E4" s="23"/>
-      <c r="F4" s="23"/>
-      <c r="G4" s="23"/>
-      <c r="H4" s="23"/>
-      <c r="I4" s="23"/>
+      <c r="A4" s="21" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="22"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="22"/>
+      <c r="G4" s="22"/>
+      <c r="H4" s="22"/>
+      <c r="I4" s="22"/>
     </row>
     <row r="5" spans="1:9" ht="15" customHeight="1">
       <c r="A5" s="1"/>
@@ -591,20 +582,20 @@
         <v>7</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E6" s="18" t="s">
         <v>8</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G6" s="11"/>
       <c r="H6" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="I6" s="21" t="s">
-        <v>14</v>
+      <c r="I6" s="19" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="15" customHeight="1">
@@ -614,7 +605,7 @@
         <v>6</v>
       </c>
       <c r="E7" s="12" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F7" s="10"/>
       <c r="G7" s="10"/>
@@ -637,25 +628,25 @@
         <v>0</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C9" s="15" t="s">
         <v>9</v>
       </c>
       <c r="D9" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="E9" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="G9" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="E9" s="16" t="s">
+      <c r="H9" s="16" t="s">
         <v>17</v>
-      </c>
-      <c r="F9" s="16" t="s">
-        <v>18</v>
-      </c>
-      <c r="G9" s="16" t="s">
-        <v>19</v>
-      </c>
-      <c r="H9" s="16" t="s">
-        <v>20</v>
       </c>
       <c r="I9" s="15" t="s">
         <v>10</v>
@@ -665,30 +656,14 @@
       <c r="A10" s="6">
         <v>1</v>
       </c>
-      <c r="B10" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="C10" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="D10" s="8">
-        <v>100</v>
-      </c>
-      <c r="E10" s="8">
-        <v>100</v>
-      </c>
-      <c r="F10" s="8">
-        <v>100</v>
-      </c>
-      <c r="G10" s="8">
-        <v>100</v>
-      </c>
-      <c r="H10" s="8">
-        <v>100</v>
-      </c>
-      <c r="I10" s="8" t="s">
-        <v>13</v>
-      </c>
+      <c r="B10" s="7"/>
+      <c r="C10" s="8"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="8"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="8"/>
+      <c r="I10" s="8"/>
     </row>
     <row r="11" spans="1:9" ht="15.75" customHeight="1">
       <c r="A11" s="6">

</xml_diff>